<commit_message>
Added mean repeatability and accuracy to the gripper tests
</commit_message>
<xml_diff>
--- a/test/GripperAccuracyRepeatabilityFlexible_test.xlsx
+++ b/test/GripperAccuracyRepeatabilityFlexible_test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rasmuslykke/Desktop/P2_Battery_Disassembly/test/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3A8D457-CF86-D94C-A4C3-502CCEF771C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A132B4AF-20C2-8D44-8502-B3E2A41FF901}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="17020" xr2:uid="{E0BA53A1-16C5-214B-8FE9-9C10E9AC2AAD}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" xr2:uid="{E0BA53A1-16C5-214B-8FE9-9C10E9AC2AAD}"/>
   </bookViews>
   <sheets>
     <sheet name="Ark1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="19">
   <si>
     <t>x</t>
   </si>
@@ -90,6 +90,12 @@
   </si>
   <si>
     <t>Flexible</t>
+  </si>
+  <si>
+    <t>Mean accuracy</t>
+  </si>
+  <si>
+    <t>Mean repeatability</t>
   </si>
 </sst>
 </file>
@@ -205,7 +211,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -228,6 +234,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -562,11 +569,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3477E26-A92D-B04D-89BF-BDDBF749FAE2}">
-  <dimension ref="A1:N13"/>
+  <dimension ref="A1:N16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="27.83203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.5" bestFit="1" customWidth="1"/>
     <col min="3" max="4" width="7" bestFit="1" customWidth="1"/>
     <col min="5" max="8" width="12.1640625" bestFit="1" customWidth="1"/>
   </cols>
@@ -1012,6 +1019,24 @@
       <c r="N13" s="7">
         <f t="shared" si="8"/>
         <v>0.26627053911388698</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="B15" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C15" s="11">
+        <f>AVERAGE(H10:H13)</f>
+        <v>1.394485084922318</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="B16" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="C16" s="7">
+        <f>AVERAGE(G10:G13)</f>
+        <v>2.0883593783517767</v>
       </c>
     </row>
   </sheetData>

</xml_diff>